<commit_message>
updating latest order history
</commit_message>
<xml_diff>
--- a/order_history_2025-03-09.xlsx
+++ b/order_history_2025-03-09.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,6 +545,126 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>20250309191435</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2025-03-09 19:14:35</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>[{'Item Name': 'bhakari', 'Price': 20.0}, {'Item Name': 'loncha', 'Price': 50.0}, {'Item Name': 'loncha', 'Price': 50.0}, {'Item Name': 'loncha', 'Price': 50.0}]</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>620</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Not Paid</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Take Away</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>20250309191456</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2025-03-09 19:14:56</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>[{'Item Name': 'bhaji', 'Price': 20.0}]</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Take Away</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>20250309192312</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2025-03-09 19:23:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>[{'Item Name': 'rice', 'Price': 30.0, 'Quantity': 1}, {'Item Name': 'rice', 'Price': 30.0, 'Quantity': 1}, {'Item Name': 'rice', 'Price': 30.0, 'Quantity': 1}]</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>90</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Not Paid</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Take Away</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>nan</t>
         </is>

</xml_diff>